<commit_message>
Fix one-candle-early flip exits; adopt best system (TRADING_RULES.md)
- flip_analysis: exit on the flip candle; user's stop/expiry rule columns;
  all 4H + 1D reports and rankings rebuilt (Stage 8o)
- Edge filter display-only: per-symbol win rates did not persist walk-forward
- Index strike = first strike at/beyond 3%; universe NIFTY + BANKNIFTY;
  journal logs index trades only; stocks shown for information (Stage 8r)
- New tests: 5-year index vs stock books, premium-free comparison (8n),
  gold GOLDBEES vs NIFTY with data cleaning (8p), Supertrend vs plain
  monthly put spread and profit-taking (8q)
- TRADING_RULES.md: current best system and scoreboard of everything tested

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exports/360ONE_full_report.xlsx
+++ b/exports/360ONE_full_report.xlsx
@@ -18,9 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,10 +53,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q75"/>
+  <dimension ref="A1:U75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,6 +512,26 @@
           <t>candles_held</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>expiry</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>reached_expiry</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>rule_trades</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>rule_wins</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -534,22 +557,22 @@
         <v>6.71</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>44585.55208333334</v>
+        <v>44586.38541666666</v>
       </c>
       <c r="H2" t="n">
-        <v>380</v>
+        <v>375.1</v>
       </c>
       <c r="I2" t="n">
         <v>379.0306861582649</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>14.16666666666667</v>
+        <v>15</v>
       </c>
       <c r="K2" t="n">
-        <v>-1.69</v>
+        <v>-2.96</v>
       </c>
       <c r="L2" t="n">
-        <v>2.25</v>
+        <v>5.64</v>
       </c>
       <c r="M2" t="n">
         <v>1.41</v>
@@ -564,7 +587,19 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>44588</v>
+      </c>
+      <c r="S2" t="b">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -591,25 +626,25 @@
         <v>10.81</v>
       </c>
       <c r="G3" s="1" t="n">
-        <v>44594.55208333334</v>
+        <v>44595.38541666666</v>
       </c>
       <c r="H3" t="n">
-        <v>405</v>
+        <v>418.25</v>
       </c>
       <c r="I3" t="n">
         <v>415.6347451255133</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>8.166666666666666</v>
+        <v>9</v>
       </c>
       <c r="K3" t="n">
-        <v>-7.97</v>
+        <v>-11.5</v>
       </c>
       <c r="L3" t="n">
-        <v>9.1</v>
+        <v>12.44</v>
       </c>
       <c r="M3" t="n">
-        <v>0.46</v>
+        <v>3.4</v>
       </c>
       <c r="N3" t="n">
         <v>4.71</v>
@@ -621,7 +656,19 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>44588</v>
+      </c>
+      <c r="S3" t="b">
+        <v>1</v>
+      </c>
+      <c r="T3" t="n">
+        <v>2</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -648,19 +695,19 @@
         <v>10.19</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>44606.55208333334</v>
+        <v>44607.38541666666</v>
       </c>
       <c r="H4" t="n">
-        <v>404.75</v>
+        <v>386.55</v>
       </c>
       <c r="I4" t="n">
         <v>387.7941611355771</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>11.16666666666667</v>
+        <v>12</v>
       </c>
       <c r="K4" t="n">
-        <v>-3.23</v>
+        <v>-7.58</v>
       </c>
       <c r="L4" t="n">
         <v>10.01</v>
@@ -678,7 +725,19 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>44616</v>
+      </c>
+      <c r="S4" t="b">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -705,19 +764,19 @@
         <v>12.2</v>
       </c>
       <c r="G5" s="1" t="n">
-        <v>44641.38541666666</v>
+        <v>44641.55208333334</v>
       </c>
       <c r="H5" t="n">
-        <v>391.55</v>
+        <v>397.75</v>
       </c>
       <c r="I5" t="n">
         <v>396.7350275012838</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>34</v>
+        <v>34.16666666666666</v>
       </c>
       <c r="K5" t="n">
-        <v>-1.29</v>
+        <v>-2.9</v>
       </c>
       <c r="L5" t="n">
         <v>7.68</v>
@@ -735,7 +794,19 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>44616</v>
+      </c>
+      <c r="S5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T5" t="n">
+        <v>2</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -762,19 +833,19 @@
         <v>9.31</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>44673.55208333334</v>
+        <v>44676.38541666666</v>
       </c>
       <c r="H6" t="n">
-        <v>437.5</v>
+        <v>424.05</v>
       </c>
       <c r="I6" t="n">
         <v>424.9266672802211</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>32</v>
+        <v>34.83333333333334</v>
       </c>
       <c r="K6" t="n">
-        <v>9.99</v>
+        <v>6.61</v>
       </c>
       <c r="L6" t="n">
         <v>2.45</v>
@@ -792,7 +863,19 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>44651</v>
+      </c>
+      <c r="S6" t="b">
+        <v>1</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -819,22 +902,22 @@
         <v>9.85</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>44683.55208333334</v>
+        <v>44685.38541666666</v>
       </c>
       <c r="H7" t="n">
-        <v>442.5</v>
+        <v>453.75</v>
       </c>
       <c r="I7" t="n">
         <v>451.0029411438092</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>7.166666666666667</v>
+        <v>9</v>
       </c>
       <c r="K7" t="n">
-        <v>-4.35</v>
+        <v>-7</v>
       </c>
       <c r="L7" t="n">
-        <v>4.82</v>
+        <v>7.89</v>
       </c>
       <c r="M7" t="n">
         <v>0.57</v>
@@ -849,7 +932,19 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>44679</v>
+      </c>
+      <c r="S7" t="b">
+        <v>1</v>
+      </c>
+      <c r="T7" t="n">
+        <v>2</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -876,28 +971,28 @@
         <v>9.890000000000001</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>44691.55208333334</v>
+        <v>44692.38541666666</v>
       </c>
       <c r="H8" t="n">
-        <v>417.5</v>
+        <v>395.85</v>
       </c>
       <c r="I8" t="n">
         <v>408.8929719805928</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>6.166666666666667</v>
+        <v>7</v>
       </c>
       <c r="K8" t="n">
-        <v>-7.99</v>
+        <v>-12.76</v>
       </c>
       <c r="L8" t="n">
-        <v>10.41</v>
+        <v>13.22</v>
       </c>
       <c r="M8" t="n">
         <v>4.99</v>
       </c>
       <c r="N8" t="n">
-        <v>4.76</v>
+        <v>6.29</v>
       </c>
       <c r="O8" t="n">
         <v>-3.28</v>
@@ -906,7 +1001,19 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>44707</v>
+      </c>
+      <c r="S8" t="b">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -933,19 +1040,19 @@
         <v>17.29</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>44741.55208333334</v>
+        <v>44742.38541666666</v>
       </c>
       <c r="H9" t="n">
-        <v>355.25</v>
+        <v>372.5</v>
       </c>
       <c r="I9" t="n">
         <v>363.6699115383219</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>49.16666666666666</v>
+        <v>50</v>
       </c>
       <c r="K9" t="n">
-        <v>10.26</v>
+        <v>5.9</v>
       </c>
       <c r="L9" t="n">
         <v>9.890000000000001</v>
@@ -963,7 +1070,19 @@
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>72</v>
+        <v>73</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>44707</v>
+      </c>
+      <c r="S9" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" t="n">
+        <v>2</v>
+      </c>
+      <c r="U9" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -990,19 +1109,19 @@
         <v>9.73</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>44830.38541666666</v>
+        <v>44830.55208333334</v>
       </c>
       <c r="H10" t="n">
-        <v>437</v>
+        <v>426.75</v>
       </c>
       <c r="I10" t="n">
         <v>432.6217746706491</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>88</v>
+        <v>88.16666666666667</v>
       </c>
       <c r="K10" t="n">
-        <v>17.32</v>
+        <v>14.56</v>
       </c>
       <c r="L10" t="n">
         <v>3.29</v>
@@ -1020,7 +1139,19 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>119</v>
+        <v>120</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>44770</v>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3</v>
+      </c>
+      <c r="U10" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1047,19 +1178,19 @@
         <v>11.32</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>44848.55208333334</v>
+        <v>44851.38541666666</v>
       </c>
       <c r="H11" t="n">
-        <v>451.25</v>
+        <v>472.4</v>
       </c>
       <c r="I11" t="n">
         <v>471.6615906963292</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>18</v>
+        <v>20.83333333333333</v>
       </c>
       <c r="K11" t="n">
-        <v>-5.74</v>
+        <v>-10.7</v>
       </c>
       <c r="L11" t="n">
         <v>11.31</v>
@@ -1077,7 +1208,19 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>44833</v>
+      </c>
+      <c r="S11" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" t="n">
+        <v>2</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1104,22 +1247,22 @@
         <v>9.58</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>44855.38541666666</v>
+        <v>44855.55208333334</v>
       </c>
       <c r="H12" t="n">
-        <v>456.45</v>
+        <v>433</v>
       </c>
       <c r="I12" t="n">
         <v>442.4982087940392</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>4</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="K12" t="n">
-        <v>-3.38</v>
+        <v>-8.34</v>
       </c>
       <c r="L12" t="n">
-        <v>4.93</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="M12" t="n">
         <v>0.41</v>
@@ -1134,7 +1277,19 @@
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>44861</v>
+      </c>
+      <c r="S12" t="b">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1161,28 +1316,28 @@
         <v>11.24</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>44893.55208333334</v>
+        <v>44894.38541666666</v>
       </c>
       <c r="H13" t="n">
-        <v>448</v>
+        <v>473</v>
       </c>
       <c r="I13" t="n">
         <v>463.3238544861484</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>38</v>
+        <v>38.83333333333334</v>
       </c>
       <c r="K13" t="n">
-        <v>-3.46</v>
+        <v>-9.24</v>
       </c>
       <c r="L13" t="n">
-        <v>8.83</v>
+        <v>11.09</v>
       </c>
       <c r="M13" t="n">
         <v>2.34</v>
       </c>
       <c r="N13" t="n">
-        <v>2.66</v>
+        <v>3.24</v>
       </c>
       <c r="O13" t="n">
         <v>-5.1</v>
@@ -1191,7 +1346,19 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="R13" s="3" t="n">
+        <v>44861</v>
+      </c>
+      <c r="S13" t="b">
+        <v>1</v>
+      </c>
+      <c r="T13" t="n">
+        <v>3</v>
+      </c>
+      <c r="U13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1218,19 +1385,19 @@
         <v>9.199999999999999</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>44917.55208333334</v>
+        <v>44918.38541666666</v>
       </c>
       <c r="H14" t="n">
-        <v>444.95</v>
+        <v>437.5</v>
       </c>
       <c r="I14" t="n">
         <v>438.6250575659793</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>23.16666666666667</v>
+        <v>24</v>
       </c>
       <c r="K14" t="n">
-        <v>-5.93</v>
+        <v>-7.51</v>
       </c>
       <c r="L14" t="n">
         <v>8.02</v>
@@ -1248,7 +1415,19 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>44924</v>
+      </c>
+      <c r="S14" t="b">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>1</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1275,19 +1454,19 @@
         <v>7.96</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>44944.38541666666</v>
+        <v>44944.55208333334</v>
       </c>
       <c r="H15" t="n">
-        <v>462.5</v>
+        <v>467.35</v>
       </c>
       <c r="I15" t="n">
         <v>463.8963194458137</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>26</v>
+        <v>26.16666666666667</v>
       </c>
       <c r="K15" t="n">
-        <v>-5.71</v>
+        <v>-6.82</v>
       </c>
       <c r="L15" t="n">
         <v>7.83</v>
@@ -1305,7 +1484,19 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="R15" s="3" t="n">
+        <v>44924</v>
+      </c>
+      <c r="S15" t="b">
+        <v>1</v>
+      </c>
+      <c r="T15" t="n">
+        <v>2</v>
+      </c>
+      <c r="U15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1332,28 +1523,28 @@
         <v>6.37</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>44953.55208333334</v>
+        <v>44956.38541666666</v>
       </c>
       <c r="H16" t="n">
-        <v>471.25</v>
+        <v>460</v>
       </c>
       <c r="I16" t="n">
         <v>460.7372802407178</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>9</v>
+        <v>11.83333333333333</v>
       </c>
       <c r="K16" t="n">
-        <v>0.83</v>
+        <v>-1.57</v>
       </c>
       <c r="L16" t="n">
-        <v>1.68</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="M16" t="n">
-        <v>0.05</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="N16" t="n">
-        <v>1.79</v>
+        <v>2.39</v>
       </c>
       <c r="O16" t="n">
         <v>2.15</v>
@@ -1362,7 +1553,19 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>44951</v>
+      </c>
+      <c r="S16" t="b">
+        <v>1</v>
+      </c>
+      <c r="T16" t="n">
+        <v>2</v>
+      </c>
+      <c r="U16" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1389,19 +1592,19 @@
         <v>6.23</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>45082.55208333334</v>
+        <v>45083.38541666666</v>
       </c>
       <c r="H17" t="n">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="I17" t="n">
         <v>425.2303291252343</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>126.1666666666667</v>
+        <v>127</v>
       </c>
       <c r="K17" t="n">
-        <v>8.699999999999999</v>
+        <v>7.17</v>
       </c>
       <c r="L17" t="n">
         <v>6.51</v>
@@ -1419,7 +1622,19 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>168</v>
+        <v>169</v>
+      </c>
+      <c r="R17" s="3" t="n">
+        <v>44980</v>
+      </c>
+      <c r="S17" t="b">
+        <v>1</v>
+      </c>
+      <c r="T17" t="n">
+        <v>5</v>
+      </c>
+      <c r="U17" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -1446,19 +1661,19 @@
         <v>5</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>45140.55208333334</v>
+        <v>45141.38541666666</v>
       </c>
       <c r="H18" t="n">
-        <v>503.15</v>
+        <v>489.1</v>
       </c>
       <c r="I18" t="n">
         <v>494.5875983789562</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>57.16666666666666</v>
+        <v>58</v>
       </c>
       <c r="K18" t="n">
-        <v>17.83</v>
+        <v>14.54</v>
       </c>
       <c r="L18" t="n">
         <v>2.55</v>
@@ -1476,7 +1691,19 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>82</v>
+        <v>83</v>
+      </c>
+      <c r="R18" s="3" t="n">
+        <v>45105</v>
+      </c>
+      <c r="S18" t="b">
+        <v>1</v>
+      </c>
+      <c r="T18" t="n">
+        <v>3</v>
+      </c>
+      <c r="U18" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1503,19 +1730,19 @@
         <v>8.58</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>45173.55208333334</v>
+        <v>45174.38541666666</v>
       </c>
       <c r="H19" t="n">
-        <v>503</v>
+        <v>518</v>
       </c>
       <c r="I19" t="n">
         <v>509.5513132699231</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>32.16666666666666</v>
+        <v>33</v>
       </c>
       <c r="K19" t="n">
-        <v>-2.84</v>
+        <v>-5.91</v>
       </c>
       <c r="L19" t="n">
         <v>6.69</v>
@@ -1533,7 +1760,19 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>45169</v>
+      </c>
+      <c r="S19" t="b">
+        <v>1</v>
+      </c>
+      <c r="T19" t="n">
+        <v>2</v>
+      </c>
+      <c r="U19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1560,19 +1799,19 @@
         <v>7.88</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>45187.38541666666</v>
+        <v>45187.55208333334</v>
       </c>
       <c r="H20" t="n">
-        <v>525.4</v>
+        <v>511.15</v>
       </c>
       <c r="I20" t="n">
         <v>515.5961843360403</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>13</v>
+        <v>13.16666666666667</v>
       </c>
       <c r="K20" t="n">
-        <v>1.43</v>
+        <v>-1.32</v>
       </c>
       <c r="L20" t="n">
         <v>2.55</v>
@@ -1590,7 +1829,19 @@
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="R20" s="3" t="n">
+        <v>45197</v>
+      </c>
+      <c r="S20" t="b">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1617,28 +1868,28 @@
         <v>11.38</v>
       </c>
       <c r="G21" s="1" t="n">
-        <v>45211.55208333334</v>
+        <v>45212.38541666666</v>
       </c>
       <c r="H21" t="n">
-        <v>510.65</v>
+        <v>537.2</v>
       </c>
       <c r="I21" t="n">
         <v>523.1789283335518</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>24</v>
+        <v>24.83333333333333</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1</v>
+        <v>-5.1</v>
       </c>
       <c r="L21" t="n">
-        <v>4.08</v>
+        <v>5.64</v>
       </c>
       <c r="M21" t="n">
         <v>1.53</v>
       </c>
       <c r="N21" t="n">
-        <v>2.79</v>
+        <v>4.96</v>
       </c>
       <c r="O21" t="n">
         <v>-2.64</v>
@@ -1647,7 +1898,19 @@
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>45197</v>
+      </c>
+      <c r="S21" t="b">
+        <v>1</v>
+      </c>
+      <c r="T21" t="n">
+        <v>2</v>
+      </c>
+      <c r="U21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1674,25 +1937,25 @@
         <v>7.5</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>45224.55208333334</v>
+        <v>45225.38541666666</v>
       </c>
       <c r="H22" t="n">
-        <v>527.55</v>
+        <v>518</v>
       </c>
       <c r="I22" t="n">
         <v>522.0683331974121</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>12.16666666666667</v>
+        <v>13</v>
       </c>
       <c r="K22" t="n">
-        <v>-1.8</v>
+        <v>-3.57</v>
       </c>
       <c r="L22" t="n">
-        <v>4.84</v>
+        <v>6.56</v>
       </c>
       <c r="M22" t="n">
-        <v>0.91</v>
+        <v>1.23</v>
       </c>
       <c r="N22" t="n">
         <v>2.98</v>
@@ -1704,7 +1967,19 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>45225</v>
+      </c>
+      <c r="S22" t="b">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1731,22 +2006,22 @@
         <v>5.74</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>45232.38541666666</v>
+        <v>45232.55208333334</v>
       </c>
       <c r="H23" t="n">
-        <v>545.3</v>
+        <v>554</v>
       </c>
       <c r="I23" t="n">
         <v>547.7218195464961</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>7</v>
+        <v>7.166666666666667</v>
       </c>
       <c r="K23" t="n">
-        <v>-5.27</v>
+        <v>-6.95</v>
       </c>
       <c r="L23" t="n">
-        <v>6.18</v>
+        <v>7.14</v>
       </c>
       <c r="M23" t="n">
         <v>1.74</v>
@@ -1761,7 +2036,19 @@
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="R23" s="3" t="n">
+        <v>45260</v>
+      </c>
+      <c r="S23" t="b">
+        <v>0</v>
+      </c>
+      <c r="T23" t="n">
+        <v>1</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1788,19 +2075,19 @@
         <v>7.02</v>
       </c>
       <c r="G24" s="1" t="n">
-        <v>45278.55208333334</v>
+        <v>45279.38541666666</v>
       </c>
       <c r="H24" t="n">
-        <v>666.5</v>
+        <v>645.65</v>
       </c>
       <c r="I24" t="n">
         <v>650.716772912541</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>46</v>
+        <v>46.83333333333334</v>
       </c>
       <c r="K24" t="n">
-        <v>20.31</v>
+        <v>16.54</v>
       </c>
       <c r="L24" t="n">
         <v>6.48</v>
@@ -1818,7 +2105,19 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="R24" s="3" t="n">
+        <v>45260</v>
+      </c>
+      <c r="S24" t="b">
+        <v>1</v>
+      </c>
+      <c r="T24" t="n">
+        <v>2</v>
+      </c>
+      <c r="U24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1845,28 +2144,28 @@
         <v>11.95</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>45287.55208333334</v>
+        <v>45288.38541666666</v>
       </c>
       <c r="H25" t="n">
-        <v>676</v>
+        <v>691.25</v>
       </c>
       <c r="I25" t="n">
         <v>687.0336038067019</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>8.166666666666666</v>
+        <v>9</v>
       </c>
       <c r="K25" t="n">
-        <v>-4.7</v>
+        <v>-7.06</v>
       </c>
       <c r="L25" t="n">
-        <v>5.09</v>
+        <v>7.46</v>
       </c>
       <c r="M25" t="n">
         <v>4.58</v>
       </c>
       <c r="N25" t="n">
-        <v>3.71</v>
+        <v>4.97</v>
       </c>
       <c r="O25" t="n">
         <v>-2.93</v>
@@ -1875,7 +2174,19 @@
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="R25" s="3" t="n">
+        <v>45288</v>
+      </c>
+      <c r="S25" t="b">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1902,22 +2213,22 @@
         <v>8.960000000000001</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>45295.38541666666</v>
+        <v>45295.55208333334</v>
       </c>
       <c r="H26" t="n">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="I26" t="n">
         <v>652.7360923220606</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>7</v>
+        <v>7.166666666666667</v>
       </c>
       <c r="K26" t="n">
-        <v>-5.24</v>
+        <v>-5.68</v>
       </c>
       <c r="L26" t="n">
-        <v>5.55</v>
+        <v>5.79</v>
       </c>
       <c r="M26" t="n">
         <v>0.23</v>
@@ -1932,7 +2243,19 @@
         <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="R26" s="3" t="n">
+        <v>45316</v>
+      </c>
+      <c r="S26" t="b">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>1</v>
+      </c>
+      <c r="U26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1959,19 +2282,19 @@
         <v>7.3</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>45329.55208333334</v>
+        <v>45330.38541666666</v>
       </c>
       <c r="H27" t="n">
-        <v>639</v>
+        <v>665.55</v>
       </c>
       <c r="I27" t="n">
         <v>649.2975253796283</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>34</v>
+        <v>34.83333333333334</v>
       </c>
       <c r="K27" t="n">
-        <v>1.99</v>
+        <v>-2.08</v>
       </c>
       <c r="L27" t="n">
         <v>5.52</v>
@@ -1989,7 +2312,19 @@
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="R27" s="3" t="n">
+        <v>45316</v>
+      </c>
+      <c r="S27" t="b">
+        <v>1</v>
+      </c>
+      <c r="T27" t="n">
+        <v>2</v>
+      </c>
+      <c r="U27" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2016,19 +2351,19 @@
         <v>9.529999999999999</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>45357.55208333334</v>
+        <v>45358.38541666666</v>
       </c>
       <c r="H28" t="n">
-        <v>702</v>
+        <v>689.75</v>
       </c>
       <c r="I28" t="n">
         <v>701.2769224580926</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>27.16666666666667</v>
+        <v>28</v>
       </c>
       <c r="K28" t="n">
-        <v>5.48</v>
+        <v>3.64</v>
       </c>
       <c r="L28" t="n">
         <v>3.68</v>
@@ -2037,7 +2372,7 @@
         <v>2.38</v>
       </c>
       <c r="N28" t="n">
-        <v>3.54</v>
+        <v>3.69</v>
       </c>
       <c r="O28" t="n">
         <v>1.41</v>
@@ -2046,7 +2381,19 @@
         <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>45351</v>
+      </c>
+      <c r="S28" t="b">
+        <v>1</v>
+      </c>
+      <c r="T28" t="n">
+        <v>2</v>
+      </c>
+      <c r="U28" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2073,19 +2420,19 @@
         <v>9.949999999999999</v>
       </c>
       <c r="G29" s="1" t="n">
-        <v>45384.38541666666</v>
+        <v>45384.55208333334</v>
       </c>
       <c r="H29" t="n">
-        <v>692.35</v>
+        <v>703</v>
       </c>
       <c r="I29" t="n">
         <v>701.1697392982994</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>26</v>
+        <v>26.16666666666667</v>
       </c>
       <c r="K29" t="n">
-        <v>-0.38</v>
+        <v>-1.92</v>
       </c>
       <c r="L29" t="n">
         <v>6.05</v>
@@ -2103,7 +2450,19 @@
         <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="R29" s="3" t="n">
+        <v>45379</v>
+      </c>
+      <c r="S29" t="b">
+        <v>1</v>
+      </c>
+      <c r="T29" t="n">
+        <v>2</v>
+      </c>
+      <c r="U29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -2130,19 +2489,19 @@
         <v>7.98</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>45418.55208333334</v>
+        <v>45419.38541666666</v>
       </c>
       <c r="H30" t="n">
-        <v>765.7</v>
+        <v>745.65</v>
       </c>
       <c r="I30" t="n">
         <v>749.262129377164</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>34</v>
+        <v>34.83333333333334</v>
       </c>
       <c r="K30" t="n">
-        <v>8.92</v>
+        <v>6.07</v>
       </c>
       <c r="L30" t="n">
         <v>1.88</v>
@@ -2160,7 +2519,19 @@
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="R30" s="3" t="n">
+        <v>45407</v>
+      </c>
+      <c r="S30" t="b">
+        <v>1</v>
+      </c>
+      <c r="T30" t="n">
+        <v>2</v>
+      </c>
+      <c r="U30" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -2187,19 +2558,19 @@
         <v>11.84</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>45434.55208333334</v>
+        <v>45435.38541666666</v>
       </c>
       <c r="H31" t="n">
-        <v>789</v>
+        <v>798.25</v>
       </c>
       <c r="I31" t="n">
         <v>794.8657427336667</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>15.16666666666667</v>
+        <v>16</v>
       </c>
       <c r="K31" t="n">
-        <v>-5.81</v>
+        <v>-7.05</v>
       </c>
       <c r="L31" t="n">
         <v>7.55</v>
@@ -2217,7 +2588,19 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>23</v>
+        <v>24</v>
+      </c>
+      <c r="R31" s="3" t="n">
+        <v>45442</v>
+      </c>
+      <c r="S31" t="b">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>1</v>
+      </c>
+      <c r="U31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -2244,28 +2627,28 @@
         <v>7.44</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>45446.55208333334</v>
+        <v>45447.38541666666</v>
       </c>
       <c r="H32" t="n">
-        <v>779</v>
+        <v>727.95</v>
       </c>
       <c r="I32" t="n">
         <v>768.8388863040212</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>11.16666666666667</v>
+        <v>12</v>
       </c>
       <c r="K32" t="n">
-        <v>-2.41</v>
+        <v>-8.81</v>
       </c>
       <c r="L32" t="n">
-        <v>4.05</v>
+        <v>13.39</v>
       </c>
       <c r="M32" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="N32" t="n">
-        <v>3.23</v>
+        <v>3.59</v>
       </c>
       <c r="O32" t="n">
         <v>2.79</v>
@@ -2274,7 +2657,19 @@
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R32" s="3" t="n">
+        <v>45442</v>
+      </c>
+      <c r="S32" t="b">
+        <v>1</v>
+      </c>
+      <c r="T32" t="n">
+        <v>2</v>
+      </c>
+      <c r="U32" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2301,28 +2696,28 @@
         <v>12.71</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>45461.55208333334</v>
+        <v>45462.38541666666</v>
       </c>
       <c r="H33" t="n">
-        <v>810</v>
+        <v>847.85</v>
       </c>
       <c r="I33" t="n">
         <v>820.1124454261839</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>14.16666666666667</v>
+        <v>15</v>
       </c>
       <c r="K33" t="n">
-        <v>-11.27</v>
+        <v>-16.47</v>
       </c>
       <c r="L33" t="n">
-        <v>12.6</v>
+        <v>18.76</v>
       </c>
       <c r="M33" t="n">
         <v>3.67</v>
       </c>
       <c r="N33" t="n">
-        <v>2.78</v>
+        <v>5.56</v>
       </c>
       <c r="O33" t="n">
         <v>-3.59</v>
@@ -2331,7 +2726,19 @@
         <v>0</v>
       </c>
       <c r="Q33" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="R33" s="3" t="n">
+        <v>45470</v>
+      </c>
+      <c r="S33" t="b">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>1</v>
+      </c>
+      <c r="U33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2358,19 +2765,19 @@
         <v>8.66</v>
       </c>
       <c r="G34" s="1" t="n">
-        <v>45505.55208333334</v>
+        <v>45506.38541666666</v>
       </c>
       <c r="H34" t="n">
-        <v>1105</v>
+        <v>1061.4</v>
       </c>
       <c r="I34" t="n">
         <v>1063.692374594539</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>43.16666666666666</v>
+        <v>44</v>
       </c>
       <c r="K34" t="n">
-        <v>30.33</v>
+        <v>25.19</v>
       </c>
       <c r="L34" t="n">
         <v>3.88</v>
@@ -2379,7 +2786,7 @@
         <v>1.33</v>
       </c>
       <c r="N34" t="n">
-        <v>4.06</v>
+        <v>4.21</v>
       </c>
       <c r="O34" t="n">
         <v>5.56</v>
@@ -2388,7 +2795,19 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="R34" s="3" t="n">
+        <v>45470</v>
+      </c>
+      <c r="S34" t="b">
+        <v>1</v>
+      </c>
+      <c r="T34" t="n">
+        <v>3</v>
+      </c>
+      <c r="U34" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -2415,22 +2834,22 @@
         <v>12.27</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>45527.55208333334</v>
+        <v>45530.38541666666</v>
       </c>
       <c r="H35" t="n">
-        <v>1086</v>
+        <v>1103.05</v>
       </c>
       <c r="I35" t="n">
         <v>1100.368272899014</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>21.16666666666667</v>
+        <v>24</v>
       </c>
       <c r="K35" t="n">
-        <v>-2.32</v>
+        <v>-3.92</v>
       </c>
       <c r="L35" t="n">
-        <v>4.85</v>
+        <v>6.45</v>
       </c>
       <c r="M35" t="n">
         <v>1.46</v>
@@ -2445,7 +2864,19 @@
         <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="R35" s="3" t="n">
+        <v>45533</v>
+      </c>
+      <c r="S35" t="b">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>1</v>
+      </c>
+      <c r="U35" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -2472,28 +2903,28 @@
         <v>6.86</v>
       </c>
       <c r="G36" s="1" t="n">
-        <v>45559.55208333334</v>
+        <v>45560.38541666666</v>
       </c>
       <c r="H36" t="n">
-        <v>1080.2</v>
+        <v>1039.65</v>
       </c>
       <c r="I36" t="n">
         <v>1045.47481008519</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>29.16666666666667</v>
+        <v>30</v>
       </c>
       <c r="K36" t="n">
-        <v>-2.07</v>
+        <v>-5.75</v>
       </c>
       <c r="L36" t="n">
-        <v>5.84</v>
+        <v>5.9</v>
       </c>
       <c r="M36" t="n">
         <v>1.16</v>
       </c>
       <c r="N36" t="n">
-        <v>3.43</v>
+        <v>4.54</v>
       </c>
       <c r="O36" t="n">
         <v>1.75</v>
@@ -2502,7 +2933,19 @@
         <v>0</v>
       </c>
       <c r="Q36" t="n">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="R36" s="3" t="n">
+        <v>45533</v>
+      </c>
+      <c r="S36" t="b">
+        <v>1</v>
+      </c>
+      <c r="T36" t="n">
+        <v>2</v>
+      </c>
+      <c r="U36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2529,19 +2972,19 @@
         <v>10.12</v>
       </c>
       <c r="G37" s="1" t="n">
-        <v>45575.55208333334</v>
+        <v>45576.38541666666</v>
       </c>
       <c r="H37" t="n">
-        <v>1025</v>
+        <v>1064.85</v>
       </c>
       <c r="I37" t="n">
         <v>1055.04119888059</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>15.16666666666667</v>
+        <v>16</v>
       </c>
       <c r="K37" t="n">
-        <v>1.41</v>
+        <v>-2.42</v>
       </c>
       <c r="L37" t="n">
         <v>6.29</v>
@@ -2559,7 +3002,19 @@
         <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="R37" s="3" t="n">
+        <v>45561</v>
+      </c>
+      <c r="S37" t="b">
+        <v>1</v>
+      </c>
+      <c r="T37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U37" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -2586,22 +3041,22 @@
         <v>11.24</v>
       </c>
       <c r="G38" s="1" t="n">
-        <v>45587.38541666666</v>
+        <v>45587.55208333334</v>
       </c>
       <c r="H38" t="n">
-        <v>1036.5</v>
+        <v>1030.2</v>
       </c>
       <c r="I38" t="n">
         <v>1031.133079079466</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>11</v>
+        <v>11.16666666666667</v>
       </c>
       <c r="K38" t="n">
-        <v>-2.66</v>
+        <v>-3.25</v>
       </c>
       <c r="L38" t="n">
-        <v>4.03</v>
+        <v>4.83</v>
       </c>
       <c r="M38" t="n">
         <v>1.54</v>
@@ -2616,7 +3071,19 @@
         <v>0</v>
       </c>
       <c r="Q38" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="R38" s="3" t="n">
+        <v>45596</v>
+      </c>
+      <c r="S38" t="b">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>1</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -2643,25 +3110,25 @@
         <v>10.21</v>
       </c>
       <c r="G39" s="1" t="n">
-        <v>45615.55208333334</v>
+        <v>45617.38541666666</v>
       </c>
       <c r="H39" t="n">
-        <v>1059</v>
+        <v>1090.55</v>
       </c>
       <c r="I39" t="n">
         <v>1089.667761491428</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>28</v>
+        <v>29.83333333333333</v>
       </c>
       <c r="K39" t="n">
-        <v>-2.8</v>
+        <v>-5.86</v>
       </c>
       <c r="L39" t="n">
-        <v>6.76</v>
+        <v>7.75</v>
       </c>
       <c r="M39" t="n">
-        <v>1.1</v>
+        <v>1.41</v>
       </c>
       <c r="N39" t="n">
         <v>4.05</v>
@@ -2673,7 +3140,19 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="R39" s="3" t="n">
+        <v>45596</v>
+      </c>
+      <c r="S39" t="b">
+        <v>1</v>
+      </c>
+      <c r="T39" t="n">
+        <v>2</v>
+      </c>
+      <c r="U39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -2700,19 +3179,19 @@
         <v>7.76</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>45664.55208333334</v>
+        <v>45665.38541666666</v>
       </c>
       <c r="H40" t="n">
-        <v>1208</v>
+        <v>1165.85</v>
       </c>
       <c r="I40" t="n">
         <v>1202.201986447673</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>47.16666666666666</v>
+        <v>48</v>
       </c>
       <c r="K40" t="n">
-        <v>10.77</v>
+        <v>6.9</v>
       </c>
       <c r="L40" t="n">
         <v>2.16</v>
@@ -2730,7 +3209,19 @@
         <v>0</v>
       </c>
       <c r="Q40" t="n">
-        <v>66</v>
+        <v>67</v>
+      </c>
+      <c r="R40" s="3" t="n">
+        <v>45624</v>
+      </c>
+      <c r="S40" t="b">
+        <v>1</v>
+      </c>
+      <c r="T40" t="n">
+        <v>3</v>
+      </c>
+      <c r="U40" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -2757,19 +3248,19 @@
         <v>10.99</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>45677.38541666666</v>
+        <v>45677.55208333334</v>
       </c>
       <c r="H41" t="n">
-        <v>1217.9</v>
+        <v>1226.3</v>
       </c>
       <c r="I41" t="n">
         <v>1223.011084784536</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>12</v>
+        <v>12.16666666666667</v>
       </c>
       <c r="K41" t="n">
-        <v>-4.46</v>
+        <v>-5.19</v>
       </c>
       <c r="L41" t="n">
         <v>5.84</v>
@@ -2787,7 +3278,19 @@
         <v>0</v>
       </c>
       <c r="Q41" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="R41" s="3" t="n">
+        <v>45687</v>
+      </c>
+      <c r="S41" t="b">
+        <v>0</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1</v>
+      </c>
+      <c r="U41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -2814,28 +3317,28 @@
         <v>10.48</v>
       </c>
       <c r="G42" s="1" t="n">
-        <v>45681.55208333334</v>
+        <v>45684.38541666666</v>
       </c>
       <c r="H42" t="n">
-        <v>1128</v>
+        <v>1073.6</v>
       </c>
       <c r="I42" t="n">
         <v>1097.794916408767</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>4</v>
+        <v>6.833333333333333</v>
       </c>
       <c r="K42" t="n">
-        <v>-8.02</v>
+        <v>-12.45</v>
       </c>
       <c r="L42" t="n">
-        <v>10.22</v>
+        <v>14.75</v>
       </c>
       <c r="M42" t="n">
         <v>0.87</v>
       </c>
       <c r="N42" t="n">
-        <v>5</v>
+        <v>5.15</v>
       </c>
       <c r="O42" t="n">
         <v>3.58</v>
@@ -2844,7 +3347,19 @@
         <v>0</v>
       </c>
       <c r="Q42" t="n">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="R42" s="3" t="n">
+        <v>45687</v>
+      </c>
+      <c r="S42" t="b">
+        <v>0</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1</v>
+      </c>
+      <c r="U42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -2871,19 +3386,19 @@
         <v>12.52</v>
       </c>
       <c r="G43" s="1" t="n">
-        <v>45709.38541666666</v>
+        <v>45709.55208333334</v>
       </c>
       <c r="H43" t="n">
-        <v>962.6</v>
+        <v>980.95</v>
       </c>
       <c r="I43" t="n">
         <v>976.437641432897</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>25</v>
+        <v>25.16666666666667</v>
       </c>
       <c r="K43" t="n">
-        <v>10.34</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L43" t="n">
         <v>4.5</v>
@@ -2901,7 +3416,19 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="R43" s="3" t="n">
+        <v>45687</v>
+      </c>
+      <c r="S43" t="b">
+        <v>1</v>
+      </c>
+      <c r="T43" t="n">
+        <v>2</v>
+      </c>
+      <c r="U43" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="44">
@@ -2928,28 +3455,28 @@
         <v>11.06</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>45723.55208333334</v>
+        <v>45726.38541666666</v>
       </c>
       <c r="H44" t="n">
-        <v>977</v>
+        <v>907.85</v>
       </c>
       <c r="I44" t="n">
         <v>927.3572994818969</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>14</v>
+        <v>16.83333333333333</v>
       </c>
       <c r="K44" t="n">
-        <v>-0.4</v>
+        <v>-7.45</v>
       </c>
       <c r="L44" t="n">
-        <v>2.53</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="M44" t="n">
         <v>1.28</v>
       </c>
       <c r="N44" t="n">
-        <v>3.32</v>
+        <v>8.5</v>
       </c>
       <c r="O44" t="n">
         <v>2.18</v>
@@ -2958,7 +3485,19 @@
         <v>0</v>
       </c>
       <c r="Q44" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="R44" s="3" t="n">
+        <v>45715</v>
+      </c>
+      <c r="S44" t="b">
+        <v>1</v>
+      </c>
+      <c r="T44" t="n">
+        <v>2</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -2985,19 +3524,19 @@
         <v>13.63</v>
       </c>
       <c r="G45" s="1" t="n">
-        <v>45736.55208333334</v>
+        <v>45737.38541666666</v>
       </c>
       <c r="H45" t="n">
-        <v>926</v>
+        <v>938.25</v>
       </c>
       <c r="I45" t="n">
         <v>926.2576533393528</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>10.16666666666667</v>
+        <v>11</v>
       </c>
       <c r="K45" t="n">
-        <v>-2</v>
+        <v>-3.35</v>
       </c>
       <c r="L45" t="n">
         <v>8.390000000000001</v>
@@ -3015,7 +3554,19 @@
         <v>1</v>
       </c>
       <c r="Q45" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R45" s="3" t="n">
+        <v>45743</v>
+      </c>
+      <c r="S45" t="b">
+        <v>0</v>
+      </c>
+      <c r="T45" t="n">
+        <v>1</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -3042,22 +3593,22 @@
         <v>9.82</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>45748.38541666666</v>
+        <v>45748.55208333334</v>
       </c>
       <c r="H46" t="n">
-        <v>905</v>
+        <v>889.9</v>
       </c>
       <c r="I46" t="n">
         <v>891.9292701389475</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>11</v>
+        <v>11.16666666666667</v>
       </c>
       <c r="K46" t="n">
-        <v>-3.54</v>
+        <v>-5.15</v>
       </c>
       <c r="L46" t="n">
-        <v>4.07</v>
+        <v>5.88</v>
       </c>
       <c r="M46" t="n">
         <v>0.9399999999999999</v>
@@ -3072,7 +3623,19 @@
         <v>0</v>
       </c>
       <c r="Q46" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>45743</v>
+      </c>
+      <c r="S46" t="b">
+        <v>1</v>
+      </c>
+      <c r="T46" t="n">
+        <v>2</v>
+      </c>
+      <c r="U46" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -3099,25 +3662,25 @@
         <v>11.39</v>
       </c>
       <c r="G47" s="1" t="n">
-        <v>45758.55208333334</v>
+        <v>45762.38541666666</v>
       </c>
       <c r="H47" t="n">
-        <v>873</v>
+        <v>932.85</v>
       </c>
       <c r="I47" t="n">
         <v>922.1045186016518</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>10</v>
+        <v>13.83333333333333</v>
       </c>
       <c r="K47" t="n">
-        <v>1.9</v>
+        <v>-4.83</v>
       </c>
       <c r="L47" t="n">
-        <v>4.71</v>
+        <v>5.73</v>
       </c>
       <c r="M47" t="n">
-        <v>1.85</v>
+        <v>3.09</v>
       </c>
       <c r="N47" t="n">
         <v>7.65</v>
@@ -3129,7 +3692,19 @@
         <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="R47" s="3" t="n">
+        <v>45771</v>
+      </c>
+      <c r="S47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1</v>
+      </c>
+      <c r="U47" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -3156,19 +3731,19 @@
         <v>14.41</v>
       </c>
       <c r="G48" s="1" t="n">
-        <v>45779.55208333334</v>
+        <v>45782.38541666666</v>
       </c>
       <c r="H48" t="n">
-        <v>949</v>
+        <v>939.35</v>
       </c>
       <c r="I48" t="n">
         <v>945.7119169557609</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>17.16666666666667</v>
+        <v>20</v>
       </c>
       <c r="K48" t="n">
-        <v>1.73</v>
+        <v>0.7</v>
       </c>
       <c r="L48" t="n">
         <v>4.06</v>
@@ -3186,7 +3761,19 @@
         <v>1</v>
       </c>
       <c r="Q48" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="R48" s="3" t="n">
+        <v>45771</v>
+      </c>
+      <c r="S48" t="b">
+        <v>1</v>
+      </c>
+      <c r="T48" t="n">
+        <v>2</v>
+      </c>
+      <c r="U48" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -3213,19 +3800,19 @@
         <v>9.710000000000001</v>
       </c>
       <c r="G49" s="1" t="n">
-        <v>45790.55208333334</v>
+        <v>45791.38541666666</v>
       </c>
       <c r="H49" t="n">
-        <v>968</v>
+        <v>983.7</v>
       </c>
       <c r="I49" t="n">
         <v>982.9621462740203</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>8.166666666666666</v>
+        <v>9</v>
       </c>
       <c r="K49" t="n">
-        <v>-3.05</v>
+        <v>-4.72</v>
       </c>
       <c r="L49" t="n">
         <v>5.39</v>
@@ -3243,7 +3830,19 @@
         <v>0</v>
       </c>
       <c r="Q49" t="n">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="R49" s="3" t="n">
+        <v>45806</v>
+      </c>
+      <c r="S49" t="b">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -3270,28 +3869,28 @@
         <v>10.15</v>
       </c>
       <c r="G50" s="1" t="n">
-        <v>45859.55208333334</v>
+        <v>45860.38541666666</v>
       </c>
       <c r="H50" t="n">
-        <v>1222</v>
+        <v>1145.3</v>
       </c>
       <c r="I50" t="n">
         <v>1157.740007202721</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>68.16666666666667</v>
+        <v>69</v>
       </c>
       <c r="K50" t="n">
-        <v>24.22</v>
+        <v>16.43</v>
       </c>
       <c r="L50" t="n">
         <v>3.45</v>
       </c>
       <c r="M50" t="n">
-        <v>1.69</v>
+        <v>3.77</v>
       </c>
       <c r="N50" t="n">
-        <v>2.72</v>
+        <v>6.31</v>
       </c>
       <c r="O50" t="n">
         <v>2.17</v>
@@ -3300,7 +3899,19 @@
         <v>0</v>
       </c>
       <c r="Q50" t="n">
-        <v>98</v>
+        <v>99</v>
+      </c>
+      <c r="R50" s="3" t="n">
+        <v>45806</v>
+      </c>
+      <c r="S50" t="b">
+        <v>1</v>
+      </c>
+      <c r="T50" t="n">
+        <v>3</v>
+      </c>
+      <c r="U50" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="51">
@@ -3327,19 +3938,19 @@
         <v>8.609999999999999</v>
       </c>
       <c r="G51" s="1" t="n">
-        <v>45888.38541666666</v>
+        <v>45888.55208333334</v>
       </c>
       <c r="H51" t="n">
-        <v>1073.7</v>
+        <v>1082</v>
       </c>
       <c r="I51" t="n">
         <v>1075.138343502455</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>28</v>
+        <v>28.16666666666667</v>
       </c>
       <c r="K51" t="n">
-        <v>6.25</v>
+        <v>5.53</v>
       </c>
       <c r="L51" t="n">
         <v>2.67</v>
@@ -3357,7 +3968,19 @@
         <v>1</v>
       </c>
       <c r="Q51" t="n">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="R51" s="3" t="n">
+        <v>45869</v>
+      </c>
+      <c r="S51" t="b">
+        <v>1</v>
+      </c>
+      <c r="T51" t="n">
+        <v>2</v>
+      </c>
+      <c r="U51" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -3384,22 +4007,22 @@
         <v>5.71</v>
       </c>
       <c r="G52" s="1" t="n">
-        <v>45897.38541666666</v>
+        <v>45897.55208333334</v>
       </c>
       <c r="H52" t="n">
-        <v>1043.1</v>
+        <v>1033.5</v>
       </c>
       <c r="I52" t="n">
         <v>1042.997323847716</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>8.833333333333334</v>
+        <v>9</v>
       </c>
       <c r="K52" t="n">
-        <v>-3.6</v>
+        <v>-4.48</v>
       </c>
       <c r="L52" t="n">
-        <v>3.7</v>
+        <v>4.98</v>
       </c>
       <c r="M52" t="n">
         <v>0.66</v>
@@ -3414,7 +4037,19 @@
         <v>0</v>
       </c>
       <c r="Q52" t="n">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="R52" s="3" t="n">
+        <v>45897</v>
+      </c>
+      <c r="S52" t="b">
+        <v>0</v>
+      </c>
+      <c r="T52" t="n">
+        <v>1</v>
+      </c>
+      <c r="U52" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -3441,22 +4076,22 @@
         <v>6.5</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>45915.38541666666</v>
+        <v>45915.55208333334</v>
       </c>
       <c r="H53" t="n">
-        <v>1076.9</v>
+        <v>1079.9</v>
       </c>
       <c r="I53" t="n">
         <v>1079.755735741162</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>17.83333333333333</v>
+        <v>18</v>
       </c>
       <c r="K53" t="n">
-        <v>-4.2</v>
+        <v>-4.49</v>
       </c>
       <c r="L53" t="n">
-        <v>4.73</v>
+        <v>4.78</v>
       </c>
       <c r="M53" t="n">
         <v>0.92</v>
@@ -3471,7 +4106,19 @@
         <v>1</v>
       </c>
       <c r="Q53" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="R53" s="3" t="n">
+        <v>45930</v>
+      </c>
+      <c r="S53" t="b">
+        <v>0</v>
+      </c>
+      <c r="T53" t="n">
+        <v>1</v>
+      </c>
+      <c r="U53" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -3498,22 +4145,22 @@
         <v>4.84</v>
       </c>
       <c r="G54" s="1" t="n">
-        <v>45922.38541666666</v>
+        <v>45922.55208333334</v>
       </c>
       <c r="H54" t="n">
-        <v>1059.2</v>
+        <v>1043.5</v>
       </c>
       <c r="I54" t="n">
         <v>1052.054482393178</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>6.833333333333333</v>
+        <v>7</v>
       </c>
       <c r="K54" t="n">
-        <v>-1.92</v>
+        <v>-3.37</v>
       </c>
       <c r="L54" t="n">
-        <v>2.15</v>
+        <v>3.49</v>
       </c>
       <c r="M54" t="n">
         <v>1.02</v>
@@ -3528,7 +4175,19 @@
         <v>0</v>
       </c>
       <c r="Q54" t="n">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="R54" s="3" t="n">
+        <v>45930</v>
+      </c>
+      <c r="S54" t="b">
+        <v>0</v>
+      </c>
+      <c r="T54" t="n">
+        <v>1</v>
+      </c>
+      <c r="U54" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -3555,22 +4214,22 @@
         <v>5.73</v>
       </c>
       <c r="G55" s="1" t="n">
-        <v>45936.55208333334</v>
+        <v>45937.38541666666</v>
       </c>
       <c r="H55" t="n">
-        <v>1057.4</v>
+        <v>1073.7</v>
       </c>
       <c r="I55" t="n">
         <v>1062.400312984279</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>14</v>
+        <v>14.83333333333333</v>
       </c>
       <c r="K55" t="n">
-        <v>-1.33</v>
+        <v>-2.89</v>
       </c>
       <c r="L55" t="n">
-        <v>2.08</v>
+        <v>3.31</v>
       </c>
       <c r="M55" t="n">
         <v>0.97</v>
@@ -3585,7 +4244,19 @@
         <v>0</v>
       </c>
       <c r="Q55" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="R55" s="3" t="n">
+        <v>45930</v>
+      </c>
+      <c r="S55" t="b">
+        <v>1</v>
+      </c>
+      <c r="T55" t="n">
+        <v>2</v>
+      </c>
+      <c r="U55" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -3612,19 +4283,19 @@
         <v>5.73</v>
       </c>
       <c r="G56" s="1" t="n">
-        <v>45960.38541666666</v>
+        <v>45960.55208333334</v>
       </c>
       <c r="H56" t="n">
-        <v>1125</v>
+        <v>1119.8</v>
       </c>
       <c r="I56" t="n">
         <v>1121.925259714254</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>23</v>
+        <v>23.16666666666667</v>
       </c>
       <c r="K56" t="n">
-        <v>4.78</v>
+        <v>4.29</v>
       </c>
       <c r="L56" t="n">
         <v>1.78</v>
@@ -3642,7 +4313,19 @@
         <v>0</v>
       </c>
       <c r="Q56" t="n">
-        <v>32</v>
+        <v>33</v>
+      </c>
+      <c r="R56" s="3" t="n">
+        <v>45958</v>
+      </c>
+      <c r="S56" t="b">
+        <v>1</v>
+      </c>
+      <c r="T56" t="n">
+        <v>2</v>
+      </c>
+      <c r="U56" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -3669,22 +4352,22 @@
         <v>5.74</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>45980.38541666666</v>
+        <v>45980.55208333334</v>
       </c>
       <c r="H57" t="n">
-        <v>1106.2</v>
+        <v>1119.1</v>
       </c>
       <c r="I57" t="n">
         <v>1118.591332625118</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>19.83333333333333</v>
+        <v>20</v>
       </c>
       <c r="K57" t="n">
-        <v>1.21</v>
+        <v>0.06</v>
       </c>
       <c r="L57" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="M57" t="n">
         <v>0.68</v>
@@ -3699,7 +4382,19 @@
         <v>0</v>
       </c>
       <c r="Q57" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="R57" s="3" t="n">
+        <v>45986</v>
+      </c>
+      <c r="S57" t="b">
+        <v>0</v>
+      </c>
+      <c r="T57" t="n">
+        <v>1</v>
+      </c>
+      <c r="U57" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -3726,19 +4421,19 @@
         <v>5.84</v>
       </c>
       <c r="G58" s="1" t="n">
-        <v>45995.38541666666</v>
+        <v>45995.55208333334</v>
       </c>
       <c r="H58" t="n">
-        <v>1131.6</v>
+        <v>1123.9</v>
       </c>
       <c r="I58" t="n">
         <v>1127.371333690995</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>14.83333333333333</v>
+        <v>15</v>
       </c>
       <c r="K58" t="n">
-        <v>1.12</v>
+        <v>0.43</v>
       </c>
       <c r="L58" t="n">
         <v>1.3</v>
@@ -3756,7 +4451,19 @@
         <v>0</v>
       </c>
       <c r="Q58" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="R58" s="3" t="n">
+        <v>45986</v>
+      </c>
+      <c r="S58" t="b">
+        <v>1</v>
+      </c>
+      <c r="T58" t="n">
+        <v>2</v>
+      </c>
+      <c r="U58" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -3783,22 +4490,22 @@
         <v>6.73</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>46013.55208333334</v>
+        <v>46014.38541666666</v>
       </c>
       <c r="H59" t="n">
-        <v>1164.7</v>
+        <v>1183.8</v>
       </c>
       <c r="I59" t="n">
         <v>1169.595897979912</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>18</v>
+        <v>18.83333333333333</v>
       </c>
       <c r="K59" t="n">
-        <v>-3.63</v>
+        <v>-5.33</v>
       </c>
       <c r="L59" t="n">
-        <v>4.9</v>
+        <v>5.45</v>
       </c>
       <c r="M59" t="n">
         <v>1.08</v>
@@ -3813,7 +4520,19 @@
         <v>0</v>
       </c>
       <c r="Q59" t="n">
-        <v>25</v>
+        <v>26</v>
+      </c>
+      <c r="R59" s="3" t="n">
+        <v>46021</v>
+      </c>
+      <c r="S59" t="b">
+        <v>0</v>
+      </c>
+      <c r="T59" t="n">
+        <v>1</v>
+      </c>
+      <c r="U59" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -3840,22 +4559,22 @@
         <v>6.69</v>
       </c>
       <c r="G60" s="1" t="n">
-        <v>46031.55208333334</v>
+        <v>46034.38541666666</v>
       </c>
       <c r="H60" t="n">
-        <v>1143.6</v>
+        <v>1127</v>
       </c>
       <c r="I60" t="n">
         <v>1137.274141507412</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>17.16666666666667</v>
+        <v>20</v>
       </c>
       <c r="K60" t="n">
-        <v>-3.4</v>
+        <v>-4.8</v>
       </c>
       <c r="L60" t="n">
-        <v>4.54</v>
+        <v>5.6</v>
       </c>
       <c r="M60" t="n">
         <v>0.83</v>
@@ -3870,7 +4589,19 @@
         <v>0</v>
       </c>
       <c r="Q60" t="n">
-        <v>26</v>
+        <v>27</v>
+      </c>
+      <c r="R60" s="3" t="n">
+        <v>46021</v>
+      </c>
+      <c r="S60" t="b">
+        <v>1</v>
+      </c>
+      <c r="T60" t="n">
+        <v>2</v>
+      </c>
+      <c r="U60" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -3897,19 +4628,19 @@
         <v>7.8</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>46099.38541666666</v>
+        <v>46099.55208333334</v>
       </c>
       <c r="H61" t="n">
-        <v>1082.2</v>
+        <v>1084.8</v>
       </c>
       <c r="I61" t="n">
         <v>1083.184376121846</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>65</v>
+        <v>65.16666666666667</v>
       </c>
       <c r="K61" t="n">
-        <v>3.98</v>
+        <v>3.74</v>
       </c>
       <c r="L61" t="n">
         <v>9.69</v>
@@ -3927,7 +4658,19 @@
         <v>0</v>
       </c>
       <c r="Q61" t="n">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="R61" s="3" t="n">
+        <v>46049</v>
+      </c>
+      <c r="S61" t="b">
+        <v>1</v>
+      </c>
+      <c r="T61" t="n">
+        <v>3</v>
+      </c>
+      <c r="U61" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="62">
@@ -3954,28 +4697,28 @@
         <v>6.88</v>
       </c>
       <c r="G62" s="1" t="n">
-        <v>46101.55208333334</v>
+        <v>46104.38541666666</v>
       </c>
       <c r="H62" t="n">
-        <v>1044.2</v>
+        <v>974.9</v>
       </c>
       <c r="I62" t="n">
         <v>1010.118845826456</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>2</v>
+        <v>4.833333333333333</v>
       </c>
       <c r="K62" t="n">
-        <v>-3.74</v>
+        <v>-10.13</v>
       </c>
       <c r="L62" t="n">
-        <v>4.63</v>
+        <v>10.22</v>
       </c>
       <c r="M62" t="n">
         <v>2.37</v>
       </c>
       <c r="N62" t="n">
-        <v>4.03</v>
+        <v>5.94</v>
       </c>
       <c r="O62" t="n">
         <v>4.44</v>
@@ -3984,7 +4727,19 @@
         <v>1</v>
       </c>
       <c r="Q62" t="n">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="R62" s="3" t="n">
+        <v>46111</v>
+      </c>
+      <c r="S62" t="b">
+        <v>0</v>
+      </c>
+      <c r="T62" t="n">
+        <v>1</v>
+      </c>
+      <c r="U62" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -4011,19 +4766,19 @@
         <v>11.69</v>
       </c>
       <c r="G63" s="1" t="n">
-        <v>46120.55208333334</v>
+        <v>46121.38541666666</v>
       </c>
       <c r="H63" t="n">
-        <v>975.5</v>
+        <v>1006.8</v>
       </c>
       <c r="I63" t="n">
         <v>993.5671888138658</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>16.16666666666667</v>
+        <v>17</v>
       </c>
       <c r="K63" t="n">
-        <v>-0.06</v>
+        <v>-3.27</v>
       </c>
       <c r="L63" t="n">
         <v>6.74</v>
@@ -4041,7 +4796,19 @@
         <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="R63" s="3" t="n">
+        <v>46111</v>
+      </c>
+      <c r="S63" t="b">
+        <v>1</v>
+      </c>
+      <c r="T63" t="n">
+        <v>2</v>
+      </c>
+      <c r="U63" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -4068,19 +4835,19 @@
         <v>10.11</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>46135.55208333334</v>
+        <v>46136.38541666666</v>
       </c>
       <c r="H64" t="n">
-        <v>1052.5</v>
+        <v>1037.8</v>
       </c>
       <c r="I64" t="n">
         <v>1043.625068729174</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>14.16666666666667</v>
+        <v>15</v>
       </c>
       <c r="K64" t="n">
-        <v>4.54</v>
+        <v>3.08</v>
       </c>
       <c r="L64" t="n">
         <v>4.19</v>
@@ -4098,7 +4865,19 @@
         <v>0</v>
       </c>
       <c r="Q64" t="n">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="R64" s="3" t="n">
+        <v>46140</v>
+      </c>
+      <c r="S64" t="b">
+        <v>0</v>
+      </c>
+      <c r="T64" t="n">
+        <v>1</v>
+      </c>
+      <c r="U64" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -4125,22 +4904,22 @@
         <v>8.58</v>
       </c>
       <c r="G65" s="1" t="n">
-        <v>46148.55208333334</v>
+        <v>46149.38541666666</v>
       </c>
       <c r="H65" t="n">
-        <v>1084.9</v>
+        <v>1109.6</v>
       </c>
       <c r="I65" t="n">
         <v>1090.2515518529</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>12.16666666666667</v>
+        <v>13</v>
       </c>
       <c r="K65" t="n">
-        <v>-4.54</v>
+        <v>-6.92</v>
       </c>
       <c r="L65" t="n">
-        <v>5.76</v>
+        <v>6.94</v>
       </c>
       <c r="M65" t="n">
         <v>0.96</v>
@@ -4155,7 +4934,19 @@
         <v>0</v>
       </c>
       <c r="Q65" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R65" s="3" t="n">
+        <v>46140</v>
+      </c>
+      <c r="S65" t="b">
+        <v>1</v>
+      </c>
+      <c r="T65" t="n">
+        <v>2</v>
+      </c>
+      <c r="U65" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -4182,22 +4973,22 @@
         <v>7.05</v>
       </c>
       <c r="G66" s="1" t="n">
-        <v>46175.55208333334</v>
+        <v>46176.38541666666</v>
       </c>
       <c r="H66" t="n">
-        <v>1087</v>
+        <v>1058.1</v>
       </c>
       <c r="I66" t="n">
         <v>1078.589887674811</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>26.16666666666667</v>
+        <v>27</v>
       </c>
       <c r="K66" t="n">
-        <v>-2.04</v>
+        <v>-4.64</v>
       </c>
       <c r="L66" t="n">
-        <v>5.21</v>
+        <v>5.44</v>
       </c>
       <c r="M66" t="n">
         <v>1.38</v>
@@ -4212,7 +5003,19 @@
         <v>0</v>
       </c>
       <c r="Q66" t="n">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="R66" s="3" t="n">
+        <v>46168</v>
+      </c>
+      <c r="S66" t="b">
+        <v>1</v>
+      </c>
+      <c r="T66" t="n">
+        <v>2</v>
+      </c>
+      <c r="U66" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -4239,28 +5042,28 @@
         <v>7.47</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>46185.55208333334</v>
+        <v>46188.38541666666</v>
       </c>
       <c r="H67" t="n">
-        <v>1094</v>
+        <v>1134.2</v>
       </c>
       <c r="I67" t="n">
         <v>1111.645856818682</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>9.166666666666666</v>
+        <v>12</v>
       </c>
       <c r="K67" t="n">
-        <v>-3.39</v>
+        <v>-7.19</v>
       </c>
       <c r="L67" t="n">
-        <v>3.87</v>
+        <v>7.2</v>
       </c>
       <c r="M67" t="n">
         <v>1.57</v>
       </c>
       <c r="N67" t="n">
-        <v>2.92</v>
+        <v>3.54</v>
       </c>
       <c r="O67" t="n">
         <v>-1.52</v>
@@ -4269,7 +5072,19 @@
         <v>0</v>
       </c>
       <c r="Q67" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R67" s="3" t="n">
+        <v>46203</v>
+      </c>
+      <c r="S67" t="b">
+        <v>0</v>
+      </c>
+      <c r="T67" t="n">
+        <v>1</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -4296,22 +5111,22 @@
         <v>7.84</v>
       </c>
       <c r="G68" s="1" t="n">
-        <v>46198.38541666666</v>
+        <v>46198.55208333334</v>
       </c>
       <c r="H68" t="n">
-        <v>1092.9</v>
+        <v>1087.8</v>
       </c>
       <c r="I68" t="n">
         <v>1090.030319699126</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>10</v>
+        <v>10.16666666666667</v>
       </c>
       <c r="K68" t="n">
-        <v>-3.64</v>
+        <v>-4.09</v>
       </c>
       <c r="L68" t="n">
-        <v>4.01</v>
+        <v>4.86</v>
       </c>
       <c r="M68" t="n">
         <v>0.31</v>
@@ -4326,7 +5141,19 @@
         <v>0</v>
       </c>
       <c r="Q68" t="n">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="R68" s="3" t="n">
+        <v>46203</v>
+      </c>
+      <c r="S68" t="b">
+        <v>0</v>
+      </c>
+      <c r="T68" t="n">
+        <v>1</v>
+      </c>
+      <c r="U68" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -4353,22 +5180,22 @@
         <v>5.01</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>46206.55208333334</v>
+        <v>46209.38541666666</v>
       </c>
       <c r="H69" t="n">
-        <v>1107.2</v>
+        <v>1128.6</v>
       </c>
       <c r="I69" t="n">
         <v>1122.486178855951</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>8</v>
+        <v>10.83333333333333</v>
       </c>
       <c r="K69" t="n">
-        <v>-1.78</v>
+        <v>-3.75</v>
       </c>
       <c r="L69" t="n">
-        <v>3.04</v>
+        <v>4.17</v>
       </c>
       <c r="M69" t="n">
         <v>0.84</v>
@@ -4383,7 +5210,19 @@
         <v>0</v>
       </c>
       <c r="Q69" t="n">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="R69" s="3" t="n">
+        <v>46203</v>
+      </c>
+      <c r="S69" t="b">
+        <v>1</v>
+      </c>
+      <c r="T69" t="n">
+        <v>2</v>
+      </c>
+      <c r="U69" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -4410,22 +5249,22 @@
         <v>6.12</v>
       </c>
       <c r="G70" s="1" t="n">
-        <v>46218.55208333334</v>
+        <v>46219.38541666666</v>
       </c>
       <c r="H70" t="n">
-        <v>1102</v>
+        <v>1078.6</v>
       </c>
       <c r="I70" t="n">
         <v>1090.515840453818</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>9.166666666666666</v>
+        <v>10</v>
       </c>
       <c r="K70" t="n">
-        <v>-2.36</v>
+        <v>-4.43</v>
       </c>
       <c r="L70" t="n">
-        <v>4.2</v>
+        <v>5.58</v>
       </c>
       <c r="M70" t="n">
         <v>1.1</v>
@@ -4440,7 +5279,19 @@
         <v>0</v>
       </c>
       <c r="Q70" t="n">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="R70" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="S70" t="b">
+        <v>0</v>
+      </c>
+      <c r="T70" t="n">
+        <v>1</v>
+      </c>
+      <c r="U70" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -4467,22 +5318,22 @@
         <v>7.24</v>
       </c>
       <c r="G71" s="1" t="n">
-        <v>46232.38541666666</v>
+        <v>46232.55208333334</v>
       </c>
       <c r="H71" t="n">
-        <v>1142.9</v>
+        <v>1162.5</v>
       </c>
       <c r="I71" t="n">
         <v>1148.372047902175</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>13</v>
+        <v>13.16666666666667</v>
       </c>
       <c r="K71" t="n">
-        <v>-5.96</v>
+        <v>-7.78</v>
       </c>
       <c r="L71" t="n">
-        <v>5.97</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="M71" t="n">
         <v>2.15</v>
@@ -4497,7 +5348,19 @@
         <v>0</v>
       </c>
       <c r="Q71" t="n">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="R71" s="3" t="n">
+        <v>46231</v>
+      </c>
+      <c r="S71" t="b">
+        <v>1</v>
+      </c>
+      <c r="T71" t="n">
+        <v>2</v>
+      </c>
+      <c r="U71" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -4524,19 +5387,19 @@
         <v>6.6</v>
       </c>
       <c r="G72" s="1" t="n">
-        <v>46266.38541666666</v>
+        <v>46266.55208333334</v>
       </c>
       <c r="H72" t="n">
-        <v>1164.3</v>
+        <v>1151.1</v>
       </c>
       <c r="I72" t="n">
         <v>1157.974632271764</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>33.83333333333334</v>
+        <v>34</v>
       </c>
       <c r="K72" t="n">
-        <v>0.15</v>
+        <v>-0.98</v>
       </c>
       <c r="L72" t="n">
         <v>3.17</v>
@@ -4554,7 +5417,19 @@
         <v>0</v>
       </c>
       <c r="Q72" t="n">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="R72" s="3" t="n">
+        <v>46259</v>
+      </c>
+      <c r="S72" t="b">
+        <v>1</v>
+      </c>
+      <c r="T72" t="n">
+        <v>2</v>
+      </c>
+      <c r="U72" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -4581,28 +5456,28 @@
         <v>5.3</v>
       </c>
       <c r="G73" s="1" t="n">
-        <v>46287.55208333334</v>
+        <v>46288.38541666666</v>
       </c>
       <c r="H73" t="n">
-        <v>1071.7</v>
+        <v>1115.1</v>
       </c>
       <c r="I73" t="n">
         <v>1099.122591891107</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>21</v>
+        <v>21.83333333333333</v>
       </c>
       <c r="K73" t="n">
-        <v>6.9</v>
+        <v>3.13</v>
       </c>
       <c r="L73" t="n">
         <v>1.77</v>
       </c>
       <c r="M73" t="n">
-        <v>0.48</v>
+        <v>2.05</v>
       </c>
       <c r="N73" t="n">
-        <v>2.08</v>
+        <v>3.28</v>
       </c>
       <c r="O73" t="n">
         <v>-1.77</v>
@@ -4611,7 +5486,19 @@
         <v>0</v>
       </c>
       <c r="Q73" t="n">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="R73" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="S73" t="b">
+        <v>0</v>
+      </c>
+      <c r="T73" t="n">
+        <v>1</v>
+      </c>
+      <c r="U73" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4638,22 +5525,22 @@
         <v>6.61</v>
       </c>
       <c r="G74" s="1" t="n">
-        <v>46290.55208333334</v>
+        <v>46293.38541666666</v>
       </c>
       <c r="H74" t="n">
-        <v>1072.5</v>
+        <v>1045.1</v>
       </c>
       <c r="I74" t="n">
         <v>1053.04215852729</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>2.166666666666667</v>
+        <v>5</v>
       </c>
       <c r="K74" t="n">
-        <v>-3.82</v>
+        <v>-6.28</v>
       </c>
       <c r="L74" t="n">
-        <v>4.74</v>
+        <v>6.42</v>
       </c>
       <c r="M74" t="n">
         <v>0.66</v>
@@ -4668,7 +5555,19 @@
         <v>0</v>
       </c>
       <c r="Q74" t="n">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="R74" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="S74" t="b">
+        <v>0</v>
+      </c>
+      <c r="T74" t="n">
+        <v>1</v>
+      </c>
+      <c r="U74" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -4719,6 +5618,14 @@
       <c r="Q75" t="n">
         <v>40</v>
       </c>
+      <c r="R75" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="S75" t="b">
+        <v>1</v>
+      </c>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6821,7 +7728,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22.6</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="6">
@@ -6831,7 +7738,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15.2</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="7">
@@ -6841,7 +7748,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>126.2</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8">
@@ -6851,7 +7758,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="9">
@@ -6861,7 +7768,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="10">
@@ -6871,7 +7778,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>45.4</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="11">
@@ -6911,7 +7818,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.57</v>
+        <v>-2.15</v>
       </c>
     </row>
     <row r="15">
@@ -6921,7 +7828,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.35</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="16">
@@ -6931,7 +7838,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-1.26</v>
+        <v>-3.85</v>
       </c>
     </row>
     <row r="17">
@@ -6941,7 +7848,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>30.33</v>
+        <v>25.19</v>
       </c>
     </row>
     <row r="18">
@@ -6951,7 +7858,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>37</v>
+        <v>27.4</v>
       </c>
     </row>
     <row r="19">
@@ -6961,7 +7868,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5.16</v>
+        <v>6.37</v>
       </c>
     </row>
     <row r="20">
@@ -6971,7 +7878,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4.74</v>
+        <v>5.88</v>
       </c>
     </row>
     <row r="21">
@@ -6981,7 +7888,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12.6</v>
+        <v>18.76</v>
       </c>
     </row>
     <row r="22">
@@ -6991,7 +7898,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23">
@@ -7001,7 +7908,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -7011,7 +7918,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1.78</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="25">
@@ -7031,7 +7938,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4.09</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="27">
@@ -7041,7 +7948,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>7.65</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="28">
@@ -7051,7 +7958,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29">

</xml_diff>